<commit_message>
chore: sync Nova upm-release-2026.10.23-01
</commit_message>
<xml_diff>
--- a/Assets/Framework/Tracks/Tracks.xlsx
+++ b/Assets/Framework/Tracks/Tracks.xlsx
@@ -1,36 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13180" activeTab="4"/>
-  </bookViews>
-  <sheets>
-    <sheet name="默认用户属性说明" sheetId="1" r:id="rId1"/>
-    <sheet name="公共事件属性说明" sheetId="2" r:id="rId2"/>
-    <sheet name="预置属性说明" sheetId="3" r:id="rId3"/>
-    <sheet name="注意事项" sheetId="4" r:id="rId4"/>
-    <sheet name="打点表-Network" sheetId="5" r:id="rId5"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'打点表-Network'!$A$1:$I$74</definedName>
-  </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" ns1:Ignorable="x15">
+  <ns0:fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <ns0:workbookPr/>
+  <ns0:bookViews>
+    <ns0:workbookView windowWidth="29100" windowHeight="13180" activeTab="4"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="默认用户属性说明" sheetId="1" ns2:id="rId1"/>
+    <ns0:sheet name="公共事件属性说明" sheetId="2" ns2:id="rId2"/>
+    <ns0:sheet name="预置属性说明" sheetId="3" ns2:id="rId3"/>
+    <ns0:sheet name="注意事项" sheetId="4" ns2:id="rId4"/>
+    <ns0:sheet name="打点表-Network" sheetId="5" ns2:id="rId5"/>
+  </ns0:sheets>
+  <ns0:definedNames>
+    <ns0:definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'打点表-Network'!$A$1:$I$74</ns0:definedName>
+  </ns0:definedNames>
+  <ns0:calcPr calcId="191029"/>
+  <ns0:extLst>
+    <ns0:ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns3:calcFeatures>
+        <ns3:feature name="microsoft.com:RD"/>
+        <ns3:feature name="microsoft.com:Single"/>
+        <ns3:feature name="microsoft.com:FV"/>
+        <ns3:feature name="microsoft.com:CNMTM"/>
+        <ns3:feature name="microsoft.com:LET_WF"/>
+        <ns3:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns3:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns3:calcFeatures>
+    </ns0:ext>
+  </ns0:extLst>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1098,836 +1098,865 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="26">
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体-简"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FF17324D"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="0"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="38">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF4EC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF17324D"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="15">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB7C7D6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB7C7D6"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB7C7D6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB7C7D6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFD9E2F3"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB7C7D6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB7C7D6"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB7C7D6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB7C7D6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB7C7D6"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB7C7D6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB7C7D6"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFB7C7D6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB7C7D6"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="10" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="11" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-  </cellStyleXfs>
-  <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
-</styleSheet>
+<ns0:styleSheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:numFmts count="0"/>
+  <ns0:fonts count="29">
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:charset val="134"/>
+      <ns0:color theme="1"/>
+      <ns0:sz val="11"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:charset val="134"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:sz val="11"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="宋体-简"/>
+      <ns0:charset val="134"/>
+      <ns0:color theme="1"/>
+      <ns0:sz val="11"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:charset val="134"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:sz val="13"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:charset val="134"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="FF17324D"/>
+      <ns0:sz val="11"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="微软雅黑"/>
+      <ns0:charset val="134"/>
+      <ns0:color theme="1"/>
+      <ns0:sz val="11"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="134"/>
+      <ns0:color theme="1"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FF0000FF"/>
+      <ns0:sz val="11"/>
+      <ns0:u val="single"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FF800080"/>
+      <ns0:sz val="11"/>
+      <ns0:u val="single"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FFFF0000"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="134"/>
+      <ns0:b val="1"/>
+      <ns0:color theme="3"/>
+      <ns0:sz val="18"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:i val="1"/>
+      <ns0:color rgb="FF7F7F7F"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="134"/>
+      <ns0:b val="1"/>
+      <ns0:color theme="3"/>
+      <ns0:sz val="15"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="134"/>
+      <ns0:b val="1"/>
+      <ns0:color theme="3"/>
+      <ns0:sz val="13"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="134"/>
+      <ns0:b val="1"/>
+      <ns0:color theme="3"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FF3F3F76"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="FF3F3F3F"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="FFFA7D00"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FFFA7D00"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:b val="1"/>
+      <ns0:color theme="1"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FF006100"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FF9C0006"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color rgb="FF9C6500"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color theme="0"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="等线"/>
+      <ns0:charset val="0"/>
+      <ns0:color theme="1"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:charset val="134"/>
+      <ns0:sz val="11"/>
+      <ns0:color theme="1"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:charset val="134"/>
+      <ns0:sz val="11"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="FFFFFFFF"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="宋体-简"/>
+      <ns0:charset val="134"/>
+      <ns0:sz val="11"/>
+      <ns0:color theme="1"/>
+    </ns0:font>
+  </ns0:fonts>
+  <ns0:fills count="38">
+    <ns0:fill>
+      <ns0:patternFill/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="gray125"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="9" tint="0.8"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF1F4E78"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFEAF4EC"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF17324D"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFD9EAF7"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFFFCC"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFCC99"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFF2F2F2"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFA5A5A5"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFC6EFCE"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFC7CE"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFEB9C"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="4"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="4" tint="0.799981688894314"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="4" tint="0.599993896298105"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="4" tint="0.399975585192419"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="5"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="5" tint="0.799981688894314"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="5" tint="0.599993896298105"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="5" tint="0.399975585192419"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="6"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="6" tint="0.799981688894314"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="6" tint="0.599993896298105"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="6" tint="0.399975585192419"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="7"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="7" tint="0.799981688894314"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="7" tint="0.599993896298105"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="7" tint="0.399975585192419"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="8"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="8" tint="0.799981688894314"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="8" tint="0.599993896298105"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="8" tint="0.399975585192419"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="9"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="9" tint="0.799981688894314"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="9" tint="0.599993896298105"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor theme="9" tint="0.399975585192419"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+  </ns0:fills>
+  <ns0:borders count="15">
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom/>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:right>
+      <ns0:top style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:top>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FFD9E2F3"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:right>
+      <ns0:top style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:top>
+      <ns0:bottom/>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:right>
+      <ns0:top/>
+      <ns0:bottom/>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:right>
+      <ns0:top/>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFB2B2B2"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FFB2B2B2"/>
+      </ns0:right>
+      <ns0:top style="thin">
+        <ns0:color rgb="FFB2B2B2"/>
+      </ns0:top>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FFB2B2B2"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom style="medium">
+        <ns0:color theme="4"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom style="medium">
+        <ns0:color theme="4" tint="0.499984740745262"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FF7F7F7F"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FF7F7F7F"/>
+      </ns0:right>
+      <ns0:top style="thin">
+        <ns0:color rgb="FF7F7F7F"/>
+      </ns0:top>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FF7F7F7F"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:left>
+      <ns0:right style="thin">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:right>
+      <ns0:top style="thin">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:top>
+      <ns0:bottom style="thin">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="double">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:left>
+      <ns0:right style="double">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:right>
+      <ns0:top style="double">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:top>
+      <ns0:bottom style="double">
+        <ns0:color rgb="FF3F3F3F"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom style="double">
+        <ns0:color rgb="FFFF8001"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top style="thin">
+        <ns0:color theme="4"/>
+      </ns0:top>
+      <ns0:bottom style="double">
+        <ns0:color theme="4"/>
+      </ns0:bottom>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color rgb="FFB7C7D6"/>
+      </ns0:left>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom/>
+      <ns0:diagonal/>
+    </ns0:border>
+  </ns0:borders>
+  <ns0:cellStyleXfs count="49">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <ns0:xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="6" fillId="7" borderId="6" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="15" fillId="8" borderId="9" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="16" fillId="9" borderId="10" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="17" fillId="9" borderId="9" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="18" fillId="10" borderId="11" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyAlignment="1">
+      <ns0:alignment vertical="center"/>
+    </ns0:xf>
+  </ns0:cellStyleXfs>
+  <ns0:cellXfs count="20">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="left" vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="left" vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="left" vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="center"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="left" vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" pivotButton="0" quotePrefix="0" applyAlignment="1">
+      <ns0:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" pivotButton="0" quotePrefix="0"/>
+    <ns0:xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" pivotButton="0" quotePrefix="0" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="28" fillId="4" borderId="1" xfId="0" pivotButton="0" quotePrefix="0" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+  </ns0:cellXfs>
+  <ns0:cellStyles count="49">
+    <ns0:cellStyle name="常规" xfId="0" builtinId="0"/>
+    <ns0:cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <ns0:cellStyle name="货币" xfId="2" builtinId="4"/>
+    <ns0:cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <ns0:cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <ns0:cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <ns0:cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <ns0:cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <ns0:cellStyle name="注释" xfId="8" builtinId="10"/>
+    <ns0:cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <ns0:cellStyle name="标题" xfId="10" builtinId="15"/>
+    <ns0:cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <ns0:cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <ns0:cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <ns0:cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <ns0:cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <ns0:cellStyle name="输入" xfId="16" builtinId="20"/>
+    <ns0:cellStyle name="输出" xfId="17" builtinId="21"/>
+    <ns0:cellStyle name="计算" xfId="18" builtinId="22"/>
+    <ns0:cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <ns0:cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <ns0:cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <ns0:cellStyle name="好" xfId="22" builtinId="26"/>
+    <ns0:cellStyle name="差" xfId="23" builtinId="27"/>
+    <ns0:cellStyle name="适中" xfId="24" builtinId="28"/>
+    <ns0:cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <ns0:cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <ns0:cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <ns0:cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <ns0:cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <ns0:cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <ns0:cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <ns0:cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <ns0:cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <ns0:cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <ns0:cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <ns0:cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <ns0:cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <ns0:cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <ns0:cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <ns0:cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <ns0:cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <ns0:cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <ns0:cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <ns0:cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <ns0:cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <ns0:cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <ns0:cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <ns0:cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  </ns0:cellStyles>
+  <ns0:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <ns0:colors/>
+</ns0:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>